<commit_message>
Remove matter/billing ID column from expense sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtKNghLZM7KdarxEtPzZZL
</commit_message>
<xml_diff>
--- a/Expense_Sheet_2026-10-09.xlsx
+++ b/Expense_Sheet_2026-10-09.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Expense Sheet" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Expense Sheet'!$A$1:$F$27</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Expense Sheet'!$A$1:$E$27</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +28,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="F9" authorId="0">
+    <comment ref="E9" authorId="0">
       <text>
         <r>
           <rPr>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t xml:space="preserve">EXPENSE REPORT</t>
   </si>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t xml:space="preserve">Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matter / Billing ID</t>
   </si>
   <si>
     <t xml:space="preserve">Amount</t>
@@ -278,7 +275,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -308,10 +305,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -595,15 +588,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -614,7 +606,6 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
@@ -662,25 +653,21 @@
       <c r="E8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="n">
         <v>46304</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="9" t="n">
+      <c r="E9" s="8" t="n">
         <v>210.11</v>
       </c>
     </row>
@@ -689,16 +676,15 @@
         <v>46304</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="8" t="n">
         <v>70.55</v>
       </c>
     </row>
@@ -707,16 +693,15 @@
         <v>46304</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="8" t="n">
         <v>13.6</v>
       </c>
     </row>
@@ -725,16 +710,15 @@
         <v>46304</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" s="8"/>
-      <c r="F12" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" s="8" t="n">
         <v>149.6</v>
       </c>
     </row>
@@ -743,104 +727,95 @@
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="10"/>
+      <c r="E13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="10"/>
+      <c r="E14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="10"/>
+      <c r="E15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="10"/>
+      <c r="E16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="10"/>
+      <c r="E17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="10"/>
+      <c r="E18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="10"/>
+      <c r="E19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="10"/>
+      <c r="E20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E21" s="11" t="s">
+      <c r="D21" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <f aca="false">SUM(E9:E20)</f>
+        <v>443.86</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="12" t="n">
-        <f aca="false">SUM(F9:F20)</f>
-        <v>443.86</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="C25" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="E25" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="14" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:E1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>

</xml_diff>